<commit_message>
Unificar notación numérica en planes de inversión
</commit_message>
<xml_diff>
--- a/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
+++ b/data/RIGI_tracker_data_final_con_proyectos_integrados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasordonez/Investigación/Tasks JCH/RIGI/rigi-dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4797E8E-89C7-AB4A-ADCC-0694C397365C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67312612-3AD8-C547-AE7C-2B7C064AE7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="68800" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1458,35 +1458,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Notas" xfId="1" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
   </cellStyles>
-  <dxfs count="32">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="29">
     <dxf>
       <font>
         <strike val="0"/>
@@ -1886,36 +1858,17 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <color rgb="FF9C0006"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF375623"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border>
@@ -1923,6 +1876,20 @@
           <color theme="1"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1988,6 +1955,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>635000</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>508000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3D984DA-D6F1-0AC1-3360-4331B5B85835}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12700000" cy="12890500"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1999,38 +2020,38 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="A1:Z41" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" headerRowBorderDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="A1:Z41" totalsRowShown="0" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27">
   <autoFilter ref="A1:Z41" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Y41">
     <sortCondition ref="D1:D41"/>
   </sortState>
   <tableColumns count="26">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="VPU" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Descripción_del_proyecto" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Proyectos de exportación estratégica de largo plazo (PEELP)" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="id_proyecto" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="empresa" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="titular_proyecto" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="CUIT" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="sector" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="subsector" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="actividad_subsector_resolución_MECON" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="provincia" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="localidad_region" dataDxfId="16"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Monto (mill. USD)" dataDxfId="15"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Monto (mill. USD) - aprobados resolución" dataDxfId="14"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Activos Computables (mill. USD)" dataDxfId="13"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Estado administrativo" dataDxfId="12"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Empleos (directos e indirectos)" dataDxfId="11"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="fecha_presentacion" dataDxfId="10"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="fecha_adhesion_rigi" dataDxfId="9"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="fecha_publicacion_bo" dataDxfId="8"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="norma_aprobacion" dataDxfId="7"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Clasificacion_preexistencia_boletin_oficial" dataDxfId="6"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Justificacion_preexistencia_boletin_oficial" dataDxfId="5"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="link_norma" dataDxfId="4"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Fuentes" dataDxfId="3"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Links_fuentes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="VPU" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Descripción_del_proyecto" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Proyectos de exportación estratégica de largo plazo (PEELP)" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="id_proyecto" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="empresa" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="titular_proyecto" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="CUIT" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="sector" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="subsector" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="actividad_subsector_resolución_MECON" dataDxfId="16"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="provincia" dataDxfId="15"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="localidad_region" dataDxfId="14"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Monto (mill. USD)" dataDxfId="13"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Monto (mill. USD) - aprobados resolución" dataDxfId="12"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Activos Computables (mill. USD)" dataDxfId="11"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Estado administrativo" dataDxfId="10"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Empleos (directos e indirectos)" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="fecha_presentacion" dataDxfId="8"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="fecha_adhesion_rigi" dataDxfId="7"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="fecha_publicacion_bo" dataDxfId="6"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="norma_aprobacion" dataDxfId="5"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Clasificacion_preexistencia_boletin_oficial" dataDxfId="4"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Justificacion_preexistencia_boletin_oficial" dataDxfId="3"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="link_norma" dataDxfId="2"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Fuentes" dataDxfId="1"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Links_fuentes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5090,8 +5111,8 @@
       <c r="H42" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="I42" s="23" t="s">
-        <v>197</v>
+      <c r="I42" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="J42" s="23"/>
       <c r="K42" s="23" t="s">

</xml_diff>